<commit_message>
reference and verse number in excel file
</commit_message>
<xml_diff>
--- a/Memory_Verses.xlsx
+++ b/Memory_Verses.xlsx
@@ -431,9 +431,140 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A2:B14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <sheetData>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Genesis 1:1 </t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Genesis 17:1 </t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Exodus 15:26 </t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Exodus 34:6 </t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Exodus </t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Leviticus 11:44 </t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Numbers 23:19 </t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Deuteronomy 7:9 </t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Deuteronomy 32:4 </t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 1 Samuel 2:2 </t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 2 Samuel 22:31 </t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 1 Kings 8:27 </t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 2 Chronicles 7:14 </t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
verses are getting printed!
</commit_message>
<xml_diff>
--- a/Memory_Verses.xlsx
+++ b/Memory_Verses.xlsx
@@ -460,7 +460,7 @@
       </c>
       <c r="C3" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">God; walk before Me and be blameless.'" </t>
+          <t xml:space="preserve">"When Abram was ninety-nine years old, the Lord appeared to Abram and said to him, 'I am Almighty God; walk before Me and be blameless.'" </t>
         </is>
       </c>
     </row>
@@ -475,7 +475,7 @@
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">brought on the Egyptians. For I am the Lord who heals you.'" </t>
+          <t xml:space="preserve">"and said, 'If you diligently heed the voice of the Lord your God and do what is right in His sight, give ear to His commandments and keep all His statutes, I will put none of the diseases on you which I have brought on the Egyptians. For I am the Lord who heals you.'" </t>
         </is>
       </c>
     </row>
@@ -490,7 +490,7 @@
       </c>
       <c r="C5" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">longsuffering, and abounding in goodness and truth, </t>
+          <t xml:space="preserve">"And the Lord passed before him and proclaimed, 'The Lord, the Lord God, merciful and gracious, longsuffering, and abounding in goodness and truth, </t>
         </is>
       </c>
     </row>
@@ -505,7 +505,7 @@
       </c>
       <c r="C6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">fourth generation. </t>
+          <t xml:space="preserve">34:7Keeping mercy for thousands, forgiving iniquity and transgression and sin, by no means clearing the guilty, visiting the iniquity of the fathers upon the children and the children’s children to the third and the fourth generation. </t>
         </is>
       </c>
     </row>
@@ -520,7 +520,7 @@
       </c>
       <c r="C7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">holy. Neither shall you defile yourselves with any creeping thing that creeps on the earth. </t>
+          <t xml:space="preserve">For I am the LORD your God. You shall therefore consecrate yourselves, and you shall be holy; for I am holy. Neither shall you defile yourselves with any creeping thing that creeps on the earth. </t>
         </is>
       </c>
     </row>
@@ -535,7 +535,7 @@
       </c>
       <c r="C8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">not do? Or has He spoken, and will He not make it good?" </t>
+          <t xml:space="preserve">God is not a man, that He should lie, Nor a son of man, that He should repent. Has He said, and will He not do? Or has He spoken, and will He not make it good?" </t>
         </is>
       </c>
     </row>
@@ -550,7 +550,7 @@
       </c>
       <c r="C9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">a thousand generations with those who love Him and keep His commandments;" </t>
+          <t xml:space="preserve">"Therefore know that the Lord your God, He is God, the faithful God who keeps covenant and mercy for a thousand generations with those who love Him and keep His commandments;" </t>
         </is>
       </c>
     </row>
@@ -565,7 +565,7 @@
       </c>
       <c r="C10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Righteous and upright is He." </t>
+          <t xml:space="preserve">"He is the Rock, His work is perfect; For all His ways are justice, A God of truth and without injustice; Righteous and upright is He." </t>
         </is>
       </c>
     </row>
@@ -610,7 +610,7 @@
       </c>
       <c r="C13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">How much less this temple which I have built!" </t>
+          <t xml:space="preserve">"But will God indeed dwell on the earth? Behold, heaven and the heaven of heavens cannot contain You. How much less this temple which I have built!" </t>
         </is>
       </c>
     </row>
@@ -625,7 +625,7 @@
       </c>
       <c r="C14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">their wicked ways, then I will hear from heaven, and I will forgive their sin and will heal their land. </t>
+          <t xml:space="preserve">their wicked ways, then I will hear from heaven, and I will forgive their sin and will heal their land. My people who are called by My name humble themselves, and pray and seek My face, and turn from their wicked ways, then I will hear from heaven, and I will forgive their sin and will heal their land. </t>
         </is>
       </c>
     </row>

</xml_diff>